<commit_message>
Redesign desktop UI using the Krona presentation palette
Introduce the burgundy and white visual system, bundled Inter typography, native SVG icons, redesigned inventory and order screens, responsive side panels, structured calculation explanations, and forecast chart tooltips. Rebuild the Windows executable and verify 38 tests plus the packaged end-to-end workflow.
</commit_message>
<xml_diff>
--- a/qa/sample_order.xlsx
+++ b/qa/sample_order.xlsx
@@ -49,7 +49,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00254E43"/>
+        <fgColor rgb="00A4002A"/>
       </patternFill>
     </fill>
   </fills>
@@ -500,7 +500,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G2" s="1" t="n"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-20T23:22:27+07:00</t>
+          <t>2026-10-21T22:01:16+07:00</t>
         </is>
       </c>
       <c r="G3" s="1" t="n"/>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>57.53934972359755</v>
+        <v>62.27934972359755</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>12</v>
@@ -647,7 +647,7 @@
         <v>5</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I5" s="1" t="n">
         <v>0</v>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>4.05</v>
+        <v>4.4</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0.8</v>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>13.13</v>
+        <v>14.2</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>1.1</v>
@@ -731,16 +731,16 @@
         <v>1</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I7" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>6110</v>
+        <v>6580</v>
       </c>
       <c r="L7" s="1" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>7.325000000000001</v>
+        <v>7.93125</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>1.4</v>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>8.376875</v>
+        <v>9.08375</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>2.8</v>
@@ -811,16 +811,16 @@
         <v>1</v>
       </c>
       <c r="H9" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>3120</v>
+        <v>3640</v>
       </c>
       <c r="L9" s="1" t="inlineStr"/>
     </row>
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>6.12</v>
+        <v>6.640000000000001</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>5.5</v>
@@ -981,7 +981,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1.460650276402447</v>
+        <v>1.720650276402452</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>2.197337430899386</v>
@@ -1006,7 +1006,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.4500000000000002</v>
+        <v>0.09999999999999964</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.1699999999999999</v>
@@ -1031,7 +1031,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.4699999999999989</v>
+        <v>0.4000000000000004</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>2.23</v>
@@ -1056,7 +1056,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.6749999999999989</v>
+        <v>0.06874999999999964</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0.3906250000000002</v>
@@ -1081,7 +1081,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.0231249999999994</v>
+        <v>0.3162499999999993</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
@@ -1106,7 +1106,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>1.08</v>
+        <v>0.5599999999999996</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
@@ -1214,13 +1214,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>101.25</v>
+        <v>110</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>84.22375974729427</v>
+        <v>96.47375944049976</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>118.2762402527057</v>
+        <v>123.5262405595002</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>164.125</v>
+        <v>177.5</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>146.6449822537801</v>
+        <v>163.3732053695606</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>181.6050177462199</v>
+        <v>191.6267946304394</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
@@ -1278,13 +1278,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>128.875</v>
+        <v>139.75</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>114.5850006426644</v>
+        <v>126.7256899199526</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>143.1649993573356</v>
+        <v>152.7743100800474</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
@@ -1308,13 +1308,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>76.5</v>
+        <v>83</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>64.86963860740136</v>
+        <v>71.48182447837598</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>88.13036139259864</v>
+        <v>94.51817552162402</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-20T23:22:27+07:00</t>
+          <t>2026-10-21T22:01:16+07:00</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Make interactive charts the main analytics workspace
Add a large sales and forecast chart with period selection, monthly comparison and fullscreen mode, plus interactive stock coverage and sales mix charts. Keep the inventory table on a separate tab. Preserve missing-data gaps and separate measured sales from forecast values. Verify 47 tests and the packaged Windows workflow.
</commit_message>
<xml_diff>
--- a/qa/sample_order.xlsx
+++ b/qa/sample_order.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-21T22:01:16+07:00</t>
+          <t>2026-10-21T22:38:31+07:00</t>
         </is>
       </c>
       <c r="G3" s="1" t="n"/>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-21T22:01:16+07:00</t>
+          <t>2026-10-21T22:38:31+07:00</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Fix seller workflows and add stock planning previews and backups
</commit_message>
<xml_diff>
--- a/qa/sample_order.xlsx
+++ b/qa/sample_order.xlsx
@@ -455,7 +455,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G2" s="1" t="n"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Тестировщик</t>
+          <t>Smoke test</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-21T22:38:31+07:00</t>
+          <t>2026-10-22T21:39:19+07:00</t>
         </is>
       </c>
       <c r="G3" s="1" t="n"/>
@@ -632,10 +632,10 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>62.27934972359755</v>
+        <v>67.00434972359754</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>5</v>
@@ -647,7 +647,7 @@
         <v>5</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I5" s="1" t="n">
         <v>0</v>
@@ -660,7 +660,7 @@
       </c>
       <c r="L5" s="1" t="inlineStr">
         <is>
-          <t>Тест ручной правки</t>
+          <t>Проверка сборки</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>4.4</v>
+        <v>4.76</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0.8</v>
@@ -691,16 +691,16 @@
         <v>1</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>1120</v>
+        <v>1400</v>
       </c>
       <c r="L6" s="1" t="inlineStr"/>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>14.2</v>
+        <v>15.27</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>1.1</v>
@@ -731,16 +731,16 @@
         <v>1</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I7" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>6580</v>
+        <v>7050</v>
       </c>
       <c r="L7" s="1" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>7.93125</v>
+        <v>8.53125</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>1.4</v>
@@ -771,16 +771,16 @@
         <v>1</v>
       </c>
       <c r="H8" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I8" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>4830</v>
+        <v>5520</v>
       </c>
       <c r="L8" s="1" t="inlineStr"/>
     </row>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>9.08375</v>
+        <v>9.774375000000001</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>2.8</v>
@@ -811,16 +811,16 @@
         <v>1</v>
       </c>
       <c r="H9" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>3640</v>
+        <v>4160</v>
       </c>
       <c r="L9" s="1" t="inlineStr"/>
     </row>
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>6.640000000000001</v>
+        <v>7.15</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>5.5</v>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>0</v>
@@ -981,10 +981,10 @@
         <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1.720650276402452</v>
+        <v>3.995650276402458</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>2.197337430899386</v>
+        <v>0.1973374308993865</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>0</v>
@@ -1006,7 +1006,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.09999999999999964</v>
+        <v>0.7400000000000002</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.1699999999999999</v>
@@ -1031,7 +1031,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.4000000000000004</v>
+        <v>0.3300000000000001</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>2.23</v>
@@ -1056,7 +1056,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.06874999999999964</v>
+        <v>0.46875</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0.3906250000000002</v>
@@ -1081,7 +1081,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.3162499999999993</v>
+        <v>0.6256249999999985</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
@@ -1106,7 +1106,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.5599999999999996</v>
+        <v>0.04999999999999982</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
@@ -1214,13 +1214,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>96.47375944049976</v>
+        <v>107.5404437881989</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>123.5262405595002</v>
+        <v>130.4595562118011</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>177.5</v>
+        <v>190.875</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>163.3732053695606</v>
+        <v>174.431683635555</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>191.6267946304394</v>
+        <v>207.318316364445</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
@@ -1278,13 +1278,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>139.75</v>
+        <v>150.375</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>126.7256899199526</v>
+        <v>133.6987612521435</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>152.7743100800474</v>
+        <v>167.0512387478565</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
@@ -1308,13 +1308,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>83</v>
+        <v>89.375</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>71.48182447837598</v>
+        <v>78.40472476300116</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>94.51817552162402</v>
+        <v>100.3452752369988</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
@@ -1440,7 +1440,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Тестировщик</t>
+          <t>Smoke test</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-21T22:38:31+07:00</t>
+          <t>2026-10-22T21:39:19+07:00</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Тест ручной правки</t>
+          <t>Проверка сборки</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add reusable adjustment reasons and faster tooltips
</commit_message>
<xml_diff>
--- a/qa/sample_order.xlsx
+++ b/qa/sample_order.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="G2" s="1" t="n"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-22T21:39:19+07:00</t>
+          <t>2026-10-23T22:10:37+07:00</t>
         </is>
       </c>
       <c r="G3" s="1" t="n"/>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>67.00434972359754</v>
+        <v>66.1889284225422</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>14</v>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>4.76</v>
+        <v>4.758000145098005</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0.8</v>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>8.53125</v>
+        <v>8.525</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>1.4</v>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>9.774375000000001</v>
+        <v>9.758125</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>2.8</v>
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>7.15</v>
+        <v>6.630385509100424</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>5.5</v>
@@ -981,10 +981,10 @@
         <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>3.995650276402458</v>
+        <v>4.811071577457795</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.1973374308993865</v>
+        <v>0.9122321056355513</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>0</v>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.7400000000000002</v>
+        <v>0.7419998549019953</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.1699999999999999</v>
+        <v>0.3895000362745011</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>0</v>
@@ -1031,7 +1031,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.3300000000000001</v>
+        <v>0.3299999999999983</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>2.23</v>
@@ -1056,7 +1056,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.46875</v>
+        <v>0.4749999999999996</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0.3906250000000002</v>
@@ -1081,7 +1081,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.6256249999999985</v>
+        <v>0.6418749999999998</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
@@ -1106,7 +1106,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.04999999999999982</v>
+        <v>0.5696144908995766</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
@@ -1156,7 +1156,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1214,17 +1214,17 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>119</v>
+        <v>118.9500036274501</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>107.5404437881989</v>
+        <v>106.7744174830715</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>130.4595562118011</v>
+        <v>131.1255897718287</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>День недели</t>
+          <t>Свежий спрос</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -1247,10 +1247,10 @@
         <v>190.875</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>174.431683635555</v>
+        <v>174.2330625637321</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>207.318316364445</v>
+        <v>207.5169374362679</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
@@ -1278,13 +1278,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>150.375</v>
+        <v>150.125</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>133.6987612521435</v>
+        <v>132.9995624217979</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>167.0512387478565</v>
+        <v>167.2504375782021</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
@@ -1308,17 +1308,17 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>89.375</v>
+        <v>82.87981886375529</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>78.40472476300116</v>
+        <v>73.68271417293668</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>100.3452752369988</v>
+        <v>92.0769235545739</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>День недели</t>
+          <t>Свежий спрос</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-22T21:39:19+07:00</t>
+          <t>2026-10-23T22:10:37+07:00</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">

</xml_diff>